<commit_message>
Add campaign tracker and PCQ MDE calculator (Excel)
- Campaign tracker: 11 campaigns across Cards/Payments/HEF/FSI
- PCQ MDE calculator: 7th decile DM test, editable inputs
- Builder scripts for both

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/campaigns/PCQ/pcq_mde_calculator.xlsx
+++ b/campaigns/PCQ/pcq_mde_calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\New_projects\cards\campaigns\PCQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89DCA40E-A0E9-4F08-98BE-30DF5C471142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E61DD97A-48FF-4AA7-BBB2-977340B6DBF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="14220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -953,7 +953,7 @@
       <c r="K22" s="12"/>
       <c r="L22" s="12"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="13">
         <v>1</v>
       </c>
@@ -992,7 +992,7 @@
         <v>Can detect &lt;0.5pp lift — GOOD</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="13">
         <v>2</v>
       </c>
@@ -1031,7 +1031,7 @@
         <v>Can detect &lt;0.5pp lift — GOOD</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="13">
         <v>3</v>
       </c>
@@ -1070,7 +1070,7 @@
         <v>Can detect &lt;0.5pp lift — GOOD</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="13">
         <v>4</v>
       </c>

</xml_diff>